<commit_message>
feat(catalog): expand beauty tech category to 30 distinct devices from dropi
</commit_message>
<xml_diff>
--- a/docs/Mesolabpro/06_Catalogo_y_Productos/02_Estudios_de_Mercado_y_Ganadores/Mesolabpro_Plantilla_Seleccion_Productos.xlsx
+++ b/docs/Mesolabpro/06_Catalogo_y_Productos/02_Estudios_de_Mercado_y_Ganadores/Mesolabpro_Plantilla_Seleccion_Productos.xlsx
@@ -581,7 +581,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AA1000"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="14.71" customWidth="1" style="39" min="1" max="1"/>
     <col width="22.57" customWidth="1" style="39" min="2" max="2"/>
@@ -808,7 +808,7 @@
         </is>
       </c>
       <c r="N2" s="16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
@@ -827,7 +827,7 @@
         <v>2</v>
       </c>
       <c r="S2" s="3" t="n">
-        <v>450</v>
+        <v>350</v>
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
@@ -840,25 +840,33 @@
         </is>
       </c>
       <c r="V2" s="3" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="W2" s="3" t="inlineStr">
         <is>
-          <t>Producto ancla. 999.000 destellos, sensor de piel. Alto ticket y margen $&gt;80k$.</t>
+          <t>999.000 destellos, sensor de contacto plano, 5 niveles.</t>
         </is>
       </c>
       <c r="X2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="Y2" s="3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z2" s="3" t="n"/>
-      <c r="AA2" s="3" t="n"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z2" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA2" s="3" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/depiladora-laser-ipl-pro</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -940,7 +948,7 @@
         <v>2</v>
       </c>
       <c r="S3" s="3" t="n">
-        <v>220</v>
+        <v>350</v>
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
@@ -953,25 +961,33 @@
         </is>
       </c>
       <c r="V3" s="3" t="n">
-        <v>9.300000000000001</v>
+        <v>9</v>
       </c>
       <c r="W3" s="3" t="inlineStr">
         <is>
-          <t>Terapia de fotones (luz roja/azul). Efecto lifting inmediato. Excelente para video UGC.</t>
+          <t>Microcorrientes EMS, radiofrecuencia bimodal y fototerapia roja/azul.</t>
         </is>
       </c>
       <c r="X3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="Y3" s="3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z3" s="3" t="n"/>
-      <c r="AA3" s="3" t="n"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z3" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA3" s="3" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/masajeador-gua-sha-radiofrecuencia-led</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1001,7 +1017,7 @@
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>Proveedor Verificado #1375642</t>
+          <t>Proveedor Verificado #55384</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -1050,10 +1066,10 @@
         <v>983</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>180</v>
+        <v>350</v>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
@@ -1066,25 +1082,33 @@
         </is>
       </c>
       <c r="V4" s="3" t="n">
-        <v>9.1</v>
+        <v>9</v>
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>Cavitación ultrasónica de 24kHz. Remueve puntos negros y células muertas. Stock masivo.</t>
+          <t>Oscilación 24 kHz, extracción de comedones sin lesión mecánica.</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z4" s="3" t="n"/>
-      <c r="AA4" s="3" t="n"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z4" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA4" s="3" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/espatula-peeling-ultrasonico</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1147,7 +1171,7 @@
         </is>
       </c>
       <c r="N5" s="16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
@@ -1166,7 +1190,7 @@
         <v>2</v>
       </c>
       <c r="S5" s="3" t="n">
-        <v>250</v>
+        <v>350</v>
       </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
@@ -1183,21 +1207,29 @@
       </c>
       <c r="W5" s="3" t="inlineStr">
         <is>
-          <t>Tratamiento anti-arrugas y definición de mandíbula. Vibración térmica 45°C. Muy viral en TikTok.</t>
+          <t>Cabezal biónico 160°, calor constante a 45°C y triple luz LED.</t>
         </is>
       </c>
       <c r="X5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="Y5" s="3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z5" s="3" t="n"/>
-      <c r="AA5" s="3" t="n"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z5" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA5" s="3" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/masajeador-cuello-papada-led</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1279,11 +1311,11 @@
         <v>2</v>
       </c>
       <c r="S6" s="3" t="n">
-        <v>550</v>
+        <v>350</v>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
@@ -1292,25 +1324,33 @@
         </is>
       </c>
       <c r="V6" s="3" t="n">
-        <v>8.9</v>
+        <v>9</v>
       </c>
       <c r="W6" s="3" t="inlineStr">
         <is>
-          <t>Nivel clínico/cabina. Cauteriza acné, estimula folículo capilar y oxigena la piel. Gran autoridad.</t>
+          <t>Gas Neón puro (naranja), acción bactericida inmediata antiacné.</t>
         </is>
       </c>
       <c r="X6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="Y6" s="3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z6" s="3" t="n"/>
-      <c r="AA6" s="3" t="n"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z6" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA6" s="3" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/equipo-alta-frecuencia-neon</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1323,31 +1363,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="12" t="n"/>
-      <c r="I7" s="14" t="n"/>
-      <c r="J7" s="14" t="n"/>
-      <c r="K7" s="15" t="n"/>
-      <c r="L7" s="14" t="n"/>
-      <c r="M7" s="3" t="n"/>
-      <c r="N7" s="16" t="n"/>
-      <c r="O7" s="3" t="n"/>
-      <c r="P7" s="3" t="n"/>
-      <c r="Q7" s="3" t="n"/>
-      <c r="R7" s="3" t="n"/>
-      <c r="S7" s="3" t="n"/>
-      <c r="T7" s="3" t="n"/>
-      <c r="U7" s="3" t="n"/>
-      <c r="V7" s="3" t="n"/>
-      <c r="W7" s="3" t="n"/>
-      <c r="X7" s="3" t="n"/>
-      <c r="Y7" s="3" t="n"/>
-      <c r="Z7" s="3" t="n"/>
-      <c r="AA7" s="3" t="n"/>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Máscaras LED y Fototerapia</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Máscara Facial Fototerapia LED 7 Colores Espectro Completo</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #43339</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>2281566</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/2281566</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="n">
+        <v>49970</v>
+      </c>
+      <c r="J7" s="14" t="n">
+        <v>129000</v>
+      </c>
+      <c r="K7" s="15">
+        <f>(J7-I7)/J7</f>
+        <v/>
+      </c>
+      <c r="L7" s="14">
+        <f>J7-I7</f>
+        <v/>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N7" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q7" s="3" t="n">
+        <v>379</v>
+      </c>
+      <c r="R7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="S7" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V7" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="W7" s="3" t="inlineStr">
+        <is>
+          <t>7 longitudes de onda, rejuvenecimiento celular y control de sebo.</t>
+        </is>
+      </c>
+      <c r="X7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y7" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA7" s="3" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/mascara-led-fototerapia-7-colores</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1360,31 +1484,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="19" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="17" t="n"/>
-      <c r="I8" s="14" t="n"/>
-      <c r="J8" s="14" t="n"/>
-      <c r="K8" s="15" t="n"/>
-      <c r="L8" s="14" t="n"/>
-      <c r="M8" s="3" t="n"/>
-      <c r="N8" s="16" t="n"/>
-      <c r="O8" s="3" t="n"/>
-      <c r="P8" s="3" t="n"/>
-      <c r="Q8" s="3" t="n"/>
-      <c r="R8" s="3" t="n"/>
-      <c r="S8" s="3" t="n"/>
-      <c r="T8" s="3" t="n"/>
-      <c r="U8" s="3" t="n"/>
-      <c r="V8" s="3" t="n"/>
-      <c r="W8" s="3" t="n"/>
-      <c r="X8" s="3" t="n"/>
-      <c r="Y8" s="3" t="n"/>
-      <c r="Z8" s="3" t="n"/>
-      <c r="AA8" s="3" t="n"/>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Dermapen y Microneedling</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Dermapen Eléctrico Auto-Microneedling Profesional</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #36223</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>1752995</t>
+        </is>
+      </c>
+      <c r="H8" s="17" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/1752995</t>
+        </is>
+      </c>
+      <c r="I8" s="14" t="n">
+        <v>70000</v>
+      </c>
+      <c r="J8" s="14" t="n">
+        <v>149000</v>
+      </c>
+      <c r="K8" s="15">
+        <f>(J8-I8)/J8</f>
+        <v/>
+      </c>
+      <c r="L8" s="14">
+        <f>J8-I8</f>
+        <v/>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N8" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="n">
+        <v>175</v>
+      </c>
+      <c r="R8" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="S8" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="T8" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V8" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="W8" s="3" t="inlineStr">
+        <is>
+          <t>Profundidad regulable 0.25mm a 2.5mm, 5 velocidades de punción.</t>
+        </is>
+      </c>
+      <c r="X8" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y8" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z8" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA8" s="3" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/dermapen-electrico-microneedling-profesional</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1397,31 +1605,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="18" t="n"/>
-      <c r="I9" s="14" t="n"/>
-      <c r="J9" s="14" t="n"/>
-      <c r="K9" s="15" t="n"/>
-      <c r="L9" s="14" t="n"/>
-      <c r="M9" s="3" t="n"/>
-      <c r="N9" s="16" t="n"/>
-      <c r="O9" s="3" t="n"/>
-      <c r="P9" s="3" t="n"/>
-      <c r="Q9" s="3" t="n"/>
-      <c r="R9" s="3" t="n"/>
-      <c r="S9" s="3" t="n"/>
-      <c r="T9" s="3" t="n"/>
-      <c r="U9" s="3" t="n"/>
-      <c r="V9" s="3" t="n"/>
-      <c r="W9" s="3" t="n"/>
-      <c r="X9" s="3" t="n"/>
-      <c r="Y9" s="3" t="n"/>
-      <c r="Z9" s="3" t="n"/>
-      <c r="AA9" s="3" t="n"/>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Vaporizadores y Saunas Faciales</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Vaporizador Facial Iónico con Nano-Niebla Térmica</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #32016</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>1192987</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/1192987</t>
+        </is>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>45000</v>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>99000</v>
+      </c>
+      <c r="K9" s="15">
+        <f>(J9-I9)/J9</f>
+        <v/>
+      </c>
+      <c r="L9" s="14">
+        <f>J9-I9</f>
+        <v/>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N9" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q9" s="3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="R9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="S9" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="T9" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U9" s="3" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V9" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="W9" s="3" t="inlineStr">
+        <is>
+          <t>Nano-iones térmicos, hidratación celular profunda y apertura de poros.</t>
+        </is>
+      </c>
+      <c r="X9" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y9" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z9" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA9" s="3" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/vaporizador-facial-ionico-nano-niebla</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1434,31 +1726,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="20" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="12" t="n"/>
-      <c r="I10" s="14" t="n"/>
-      <c r="J10" s="14" t="n"/>
-      <c r="K10" s="15" t="n"/>
-      <c r="L10" s="14" t="n"/>
-      <c r="M10" s="3" t="n"/>
-      <c r="N10" s="16" t="n"/>
-      <c r="O10" s="3" t="n"/>
-      <c r="P10" s="3" t="n"/>
-      <c r="Q10" s="3" t="n"/>
-      <c r="R10" s="3" t="n"/>
-      <c r="S10" s="3" t="n"/>
-      <c r="T10" s="3" t="n"/>
-      <c r="U10" s="3" t="n"/>
-      <c r="V10" s="3" t="n"/>
-      <c r="W10" s="3" t="n"/>
-      <c r="X10" s="3" t="n"/>
-      <c r="Y10" s="3" t="n"/>
-      <c r="Z10" s="3" t="n"/>
-      <c r="AA10" s="3" t="n"/>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Extractores de Poros y Succión</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Extractor Hidrofacial por Microburbujas y Succión al Vacío</t>
+        </is>
+      </c>
+      <c r="F10" s="20" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #43728</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>1824329</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/1824329</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="n">
+        <v>28000</v>
+      </c>
+      <c r="J10" s="14" t="n">
+        <v>89000</v>
+      </c>
+      <c r="K10" s="15">
+        <f>(J10-I10)/J10</f>
+        <v/>
+      </c>
+      <c r="L10" s="14">
+        <f>J10-I10</f>
+        <v/>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N10" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q10" s="3" t="n">
+        <v>218</v>
+      </c>
+      <c r="R10" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="S10" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="T10" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U10" s="3" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="W10" s="3" t="inlineStr">
+        <is>
+          <t>Hidrodermoabrasión con doble tanque independiente y 6 boquillas.</t>
+        </is>
+      </c>
+      <c r="X10" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y10" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z10" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA10" s="3" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/extractor-hidrofacial-microburbujas-vacio</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1471,31 +1847,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="8" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="18" t="n"/>
-      <c r="I11" s="14" t="n"/>
-      <c r="J11" s="14" t="n"/>
-      <c r="K11" s="15" t="n"/>
-      <c r="L11" s="14" t="n"/>
-      <c r="M11" s="3" t="n"/>
-      <c r="N11" s="3" t="n"/>
-      <c r="O11" s="3" t="n"/>
-      <c r="P11" s="3" t="n"/>
-      <c r="Q11" s="3" t="n"/>
-      <c r="R11" s="3" t="n"/>
-      <c r="S11" s="3" t="n"/>
-      <c r="T11" s="3" t="n"/>
-      <c r="U11" s="3" t="n"/>
-      <c r="V11" s="3" t="n"/>
-      <c r="W11" s="3" t="n"/>
-      <c r="X11" s="3" t="n"/>
-      <c r="Y11" s="3" t="n"/>
-      <c r="Z11" s="3" t="n"/>
-      <c r="AA11" s="3" t="n"/>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Cavitación y Reducción Corporal</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Equipo Cavitador Ultrasónico y EMS Corporal 3 en 1</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #36082</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>788821</t>
+        </is>
+      </c>
+      <c r="H11" s="18" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/788821</t>
+        </is>
+      </c>
+      <c r="I11" s="14" t="n">
+        <v>52000</v>
+      </c>
+      <c r="J11" s="14" t="n">
+        <v>139000</v>
+      </c>
+      <c r="K11" s="15">
+        <f>(J11-I11)/J11</f>
+        <v/>
+      </c>
+      <c r="L11" s="14">
+        <f>J11-I11</f>
+        <v/>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q11" s="3" t="n">
+        <v>249</v>
+      </c>
+      <c r="R11" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="S11" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="T11" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U11" s="3" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V11" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="W11" s="3" t="inlineStr">
+        <is>
+          <t>Ultrasonido 1 MHz, infrarrojo térmico y gimnasia pasiva EMS.</t>
+        </is>
+      </c>
+      <c r="X11" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y11" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z11" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA11" s="3" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/cavitador-ultrasonico-ems-corporal-3en1</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1508,31 +1968,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="8" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="12" t="n"/>
-      <c r="I12" s="14" t="n"/>
-      <c r="J12" s="14" t="n"/>
-      <c r="K12" s="15" t="n"/>
-      <c r="L12" s="14" t="n"/>
-      <c r="M12" s="3" t="n"/>
-      <c r="N12" s="3" t="n"/>
-      <c r="O12" s="3" t="n"/>
-      <c r="P12" s="3" t="n"/>
-      <c r="Q12" s="3" t="n"/>
-      <c r="R12" s="3" t="n"/>
-      <c r="S12" s="3" t="n"/>
-      <c r="T12" s="3" t="n"/>
-      <c r="U12" s="3" t="n"/>
-      <c r="V12" s="3" t="n"/>
-      <c r="W12" s="3" t="n"/>
-      <c r="X12" s="3" t="n"/>
-      <c r="Y12" s="3" t="n"/>
-      <c r="Z12" s="3" t="n"/>
-      <c r="AA12" s="3" t="n"/>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Plasma Pen y Cauterizadores</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Lápiz Cauterizador Plasma Pen Recargable</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #197931</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>1982303</t>
+        </is>
+      </c>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/1982303</t>
+        </is>
+      </c>
+      <c r="I12" s="14" t="n">
+        <v>42000</v>
+      </c>
+      <c r="J12" s="14" t="n">
+        <v>99000</v>
+      </c>
+      <c r="K12" s="15">
+        <f>(J12-I12)/J12</f>
+        <v/>
+      </c>
+      <c r="L12" s="14">
+        <f>J12-I12</f>
+        <v/>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="R12" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="S12" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U12" s="3" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V12" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="W12" s="3" t="inlineStr">
+        <is>
+          <t>Descarga de microplasma de baja temperatura, 9 niveles.</t>
+        </is>
+      </c>
+      <c r="X12" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y12" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z12" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA12" s="3" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/plasma-pen-cauterizador-recargable</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1545,31 +2089,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="17" t="n"/>
-      <c r="I13" s="14" t="n"/>
-      <c r="J13" s="14" t="n"/>
-      <c r="K13" s="15" t="n"/>
-      <c r="L13" s="14" t="n"/>
-      <c r="M13" s="3" t="n"/>
-      <c r="N13" s="3" t="n"/>
-      <c r="O13" s="3" t="n"/>
-      <c r="P13" s="3" t="n"/>
-      <c r="Q13" s="3" t="n"/>
-      <c r="R13" s="3" t="n"/>
-      <c r="S13" s="3" t="n"/>
-      <c r="T13" s="3" t="n"/>
-      <c r="U13" s="3" t="n"/>
-      <c r="V13" s="3" t="n"/>
-      <c r="W13" s="3" t="n"/>
-      <c r="X13" s="3" t="n"/>
-      <c r="Y13" s="3" t="n"/>
-      <c r="Z13" s="3" t="n"/>
-      <c r="AA13" s="3" t="n"/>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Cepillos y Limpiadores Sónicos</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Cepillo Limpiador Facial Giratorio 5 en 1 Beauty Care</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #7151</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>98860</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/98860</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="n">
+        <v>13000</v>
+      </c>
+      <c r="J13" s="14" t="n">
+        <v>59000</v>
+      </c>
+      <c r="K13" s="15">
+        <f>(J13-I13)/J13</f>
+        <v/>
+      </c>
+      <c r="L13" s="14">
+        <f>J13-I13</f>
+        <v/>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q13" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="R13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="S13" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="T13" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U13" s="3" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V13" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="W13" s="3" t="inlineStr">
+        <is>
+          <t>Sistema rotativo con 5 cabezales intercambiables de exfoliación.</t>
+        </is>
+      </c>
+      <c r="X13" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y13" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z13" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA13" s="3" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/cepillo-facial-giratorio-5en1</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1582,31 +2210,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="8" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="12" t="n"/>
-      <c r="I14" s="14" t="n"/>
-      <c r="J14" s="14" t="n"/>
-      <c r="K14" s="15" t="n"/>
-      <c r="L14" s="14" t="n"/>
-      <c r="M14" s="3" t="n"/>
-      <c r="N14" s="3" t="n"/>
-      <c r="O14" s="3" t="n"/>
-      <c r="P14" s="3" t="n"/>
-      <c r="Q14" s="3" t="n"/>
-      <c r="R14" s="3" t="n"/>
-      <c r="S14" s="3" t="n"/>
-      <c r="T14" s="3" t="n"/>
-      <c r="U14" s="3" t="n"/>
-      <c r="V14" s="3" t="n"/>
-      <c r="W14" s="3" t="n"/>
-      <c r="X14" s="3" t="n"/>
-      <c r="Y14" s="3" t="n"/>
-      <c r="Z14" s="3" t="n"/>
-      <c r="AA14" s="3" t="n"/>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Radiofrecuencia y Electroporación</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Dispositivo Radiofrecuencia Facial Tripolar con Fototerapia LED</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #394103</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>1851775</t>
+        </is>
+      </c>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/1851775</t>
+        </is>
+      </c>
+      <c r="I14" s="14" t="n">
+        <v>55900</v>
+      </c>
+      <c r="J14" s="14" t="n">
+        <v>129000</v>
+      </c>
+      <c r="K14" s="15">
+        <f>(J14-I14)/J14</f>
+        <v/>
+      </c>
+      <c r="L14" s="14">
+        <f>J14-I14</f>
+        <v/>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="n">
+        <v>654</v>
+      </c>
+      <c r="R14" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="S14" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U14" s="3" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V14" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="W14" s="3" t="inlineStr">
+        <is>
+          <t>Ondas electromagnéticas tripolares y 5 terapias LED dérmicas.</t>
+        </is>
+      </c>
+      <c r="X14" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y14" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z14" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA14" s="3" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/radiofrecuencia-facial-tripolar-led</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1619,31 +2331,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="8" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="3" t="n"/>
-      <c r="H15" s="12" t="n"/>
-      <c r="I15" s="14" t="n"/>
-      <c r="J15" s="14" t="n"/>
-      <c r="K15" s="15" t="n"/>
-      <c r="L15" s="14" t="n"/>
-      <c r="M15" s="3" t="n"/>
-      <c r="N15" s="3" t="n"/>
-      <c r="O15" s="3" t="n"/>
-      <c r="P15" s="3" t="n"/>
-      <c r="Q15" s="3" t="n"/>
-      <c r="R15" s="3" t="n"/>
-      <c r="S15" s="3" t="n"/>
-      <c r="T15" s="3" t="n"/>
-      <c r="U15" s="3" t="n"/>
-      <c r="V15" s="3" t="n"/>
-      <c r="W15" s="3" t="n"/>
-      <c r="X15" s="3" t="n"/>
-      <c r="Y15" s="3" t="n"/>
-      <c r="Z15" s="3" t="n"/>
-      <c r="AA15" s="3" t="n"/>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Alta Frecuencia y Microcorrientes</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Derma Wand Pro Tonificador Facial por Alta Frecuencia</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #144205</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>1682676</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/1682676</t>
+        </is>
+      </c>
+      <c r="I15" s="14" t="n">
+        <v>37000</v>
+      </c>
+      <c r="J15" s="14" t="n">
+        <v>99000</v>
+      </c>
+      <c r="K15" s="15">
+        <f>(J15-I15)/J15</f>
+        <v/>
+      </c>
+      <c r="L15" s="14">
+        <f>J15-I15</f>
+        <v/>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q15" s="3" t="n">
+        <v>382</v>
+      </c>
+      <c r="R15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="S15" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="T15" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U15" s="3" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V15" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="W15" s="3" t="inlineStr">
+        <is>
+          <t>Microcorrientes a 100.000 ciclos/seg con liberación de oxígeno.</t>
+        </is>
+      </c>
+      <c r="X15" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y15" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z15" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA15" s="3" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/derma-wand-pro-tonificador-facial</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1656,31 +2452,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="8" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="12" t="n"/>
-      <c r="I16" s="14" t="n"/>
-      <c r="J16" s="14" t="n"/>
-      <c r="K16" s="15" t="n"/>
-      <c r="L16" s="14" t="n"/>
-      <c r="M16" s="3" t="n"/>
-      <c r="N16" s="3" t="n"/>
-      <c r="O16" s="3" t="n"/>
-      <c r="P16" s="3" t="n"/>
-      <c r="Q16" s="3" t="n"/>
-      <c r="R16" s="3" t="n"/>
-      <c r="S16" s="3" t="n"/>
-      <c r="T16" s="3" t="n"/>
-      <c r="U16" s="3" t="n"/>
-      <c r="V16" s="3" t="n"/>
-      <c r="W16" s="3" t="n"/>
-      <c r="X16" s="3" t="n"/>
-      <c r="Y16" s="3" t="n"/>
-      <c r="Z16" s="3" t="n"/>
-      <c r="AA16" s="3" t="n"/>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Aparatología Capilar</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Cepillo Masajeador Capilar Eléctrico 3D Fototerapia</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #228310</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>2097027</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/2097027</t>
+        </is>
+      </c>
+      <c r="I16" s="14" t="n">
+        <v>32000</v>
+      </c>
+      <c r="J16" s="14" t="n">
+        <v>89000</v>
+      </c>
+      <c r="K16" s="15">
+        <f>(J16-I16)/J16</f>
+        <v/>
+      </c>
+      <c r="L16" s="14">
+        <f>J16-I16</f>
+        <v/>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q16" s="3" t="n">
+        <v>4976</v>
+      </c>
+      <c r="R16" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="S16" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="T16" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U16" s="3" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V16" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="W16" s="3" t="inlineStr">
+        <is>
+          <t>Masaje tridimensional 3D con fototerapia roja y reactivación folicular.</t>
+        </is>
+      </c>
+      <c r="X16" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y16" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z16" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA16" s="3" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/cepillo-masajeador-capilar-electrico-3d</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1693,18 +2573,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="8" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="3" t="n"/>
-      <c r="H17" s="17" t="n"/>
-      <c r="I17" s="14" t="n"/>
-      <c r="J17" s="14" t="n"/>
-      <c r="K17" s="15" t="n"/>
-      <c r="L17" s="14" t="n"/>
-      <c r="M17" s="3" t="n"/>
-      <c r="N17" s="3" t="n"/>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Aparatología Capilar</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Cepillo Masajeador Capilar con Nano Spray de Iones</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #141975</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>2222902</t>
+        </is>
+      </c>
+      <c r="H17" s="17" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/2222902</t>
+        </is>
+      </c>
+      <c r="I17" s="14" t="n">
+        <v>23000</v>
+      </c>
+      <c r="J17" s="14" t="n">
+        <v>69000</v>
+      </c>
+      <c r="K17" s="15">
+        <f>(J17-I17)/J17</f>
+        <v/>
+      </c>
+      <c r="L17" s="14">
+        <f>J17-I17</f>
+        <v/>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O17" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P17" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q17" s="0" t="n">
+        <v>206</v>
+      </c>
+      <c r="R17" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="S17" s="0" t="n">
+        <v>350</v>
+      </c>
+      <c r="T17" s="0" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U17" s="0" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V17" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="W17" s="0" t="inlineStr">
+        <is>
+          <t>Nebulización ultrasónica de lociones capilares y desenredo anti-frizz.</t>
+        </is>
+      </c>
+      <c r="X17" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y17" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z17" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA17" s="0" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/cepillo-capilar-nano-spray-iones</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1717,18 +2694,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
-      <c r="E18" s="8" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="3" t="n"/>
-      <c r="H18" s="17" t="n"/>
-      <c r="I18" s="14" t="n"/>
-      <c r="J18" s="14" t="n"/>
-      <c r="K18" s="15" t="n"/>
-      <c r="L18" s="14" t="n"/>
-      <c r="M18" s="3" t="n"/>
-      <c r="N18" s="3" t="n"/>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Ojos y Pestañas Tech</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Rizador Térmico de Pestañas Eléctrico con Termorregulación</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #894235</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>2168876</t>
+        </is>
+      </c>
+      <c r="H18" s="17" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/2168876</t>
+        </is>
+      </c>
+      <c r="I18" s="14" t="n">
+        <v>13000</v>
+      </c>
+      <c r="J18" s="14" t="n">
+        <v>49000</v>
+      </c>
+      <c r="K18" s="15">
+        <f>(J18-I18)/J18</f>
+        <v/>
+      </c>
+      <c r="L18" s="14">
+        <f>J18-I18</f>
+        <v/>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O18" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P18" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q18" s="0" t="n">
+        <v>145</v>
+      </c>
+      <c r="R18" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="S18" s="0" t="n">
+        <v>350</v>
+      </c>
+      <c r="T18" s="0" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U18" s="0" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V18" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="W18" s="0" t="inlineStr">
+        <is>
+          <t>Calor constante a 65-85°C con almohadilla de silicona termoactiva.</t>
+        </is>
+      </c>
+      <c r="X18" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y18" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z18" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA18" s="0" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/rizador-termico-pestanas-electrico</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1741,18 +2815,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="8" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="18" t="n"/>
-      <c r="I19" s="14" t="n"/>
-      <c r="J19" s="14" t="n"/>
-      <c r="K19" s="15" t="n"/>
-      <c r="L19" s="14" t="n"/>
-      <c r="M19" s="3" t="n"/>
-      <c r="N19" s="3" t="n"/>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Depilación Láser IPL</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Depiladora Facial de Precisión y Perfilador de Cejas</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #49923</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>1965520</t>
+        </is>
+      </c>
+      <c r="H19" s="18" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/1965520</t>
+        </is>
+      </c>
+      <c r="I19" s="14" t="n">
+        <v>31980</v>
+      </c>
+      <c r="J19" s="14" t="n">
+        <v>79000</v>
+      </c>
+      <c r="K19" s="15">
+        <f>(J19-I19)/J19</f>
+        <v/>
+      </c>
+      <c r="L19" s="14">
+        <f>J19-I19</f>
+        <v/>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O19" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P19" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q19" s="0" t="n">
+        <v>1222</v>
+      </c>
+      <c r="R19" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="S19" s="0" t="n">
+        <v>350</v>
+      </c>
+      <c r="T19" s="0" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U19" s="0" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V19" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="W19" s="0" t="inlineStr">
+        <is>
+          <t>Cabezal microquirúrgico dual hipoalergénico con luz LED auxiliar.</t>
+        </is>
+      </c>
+      <c r="X19" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y19" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z19" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA19" s="0" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/depiladora-facial-cejas-recargable</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1765,18 +2936,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="8" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="17" t="n"/>
-      <c r="I20" s="14" t="n"/>
-      <c r="J20" s="14" t="n"/>
-      <c r="K20" s="15" t="n"/>
-      <c r="L20" s="14" t="n"/>
-      <c r="M20" s="3" t="n"/>
-      <c r="N20" s="3" t="n"/>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Depilación Láser IPL</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Depiladora Facial Multifunción 4 en 1 para Rostro y Cuerpo</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #32016</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>242034</t>
+        </is>
+      </c>
+      <c r="H20" s="17" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/242034</t>
+        </is>
+      </c>
+      <c r="I20" s="14" t="n">
+        <v>24000</v>
+      </c>
+      <c r="J20" s="14" t="n">
+        <v>69000</v>
+      </c>
+      <c r="K20" s="15">
+        <f>(J20-I20)/J20</f>
+        <v/>
+      </c>
+      <c r="L20" s="14">
+        <f>J20-I20</f>
+        <v/>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O20" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P20" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q20" s="0" t="n">
+        <v>676</v>
+      </c>
+      <c r="R20" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="S20" s="0" t="n">
+        <v>350</v>
+      </c>
+      <c r="T20" s="0" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U20" s="0" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V20" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="W20" s="0" t="inlineStr">
+        <is>
+          <t>Kit 4 en 1 para rostro, cejas, nariz y zona bikini sin tirones.</t>
+        </is>
+      </c>
+      <c r="X20" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y20" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z20" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA20" s="0" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/depiladora-facial-multifuncion-4en1</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="39">
       <c r="A21" s="3" t="inlineStr">
@@ -1789,18 +3057,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C21" s="7" t="n"/>
-      <c r="D21" s="7" t="n"/>
-      <c r="E21" s="8" t="n"/>
-      <c r="F21" s="10" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="17" t="n"/>
-      <c r="I21" s="14" t="n"/>
-      <c r="J21" s="14" t="n"/>
-      <c r="K21" s="15" t="n"/>
-      <c r="L21" s="14" t="n"/>
-      <c r="M21" s="3" t="n"/>
-      <c r="N21" s="3" t="n"/>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Vaporizadores y Saunas Faciales</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Sauna Facial con Inhalador Térmico Spa para Hidratación</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #49923</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>1965189</t>
+        </is>
+      </c>
+      <c r="H21" s="17" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/1965189</t>
+        </is>
+      </c>
+      <c r="I21" s="14" t="n">
+        <v>52777</v>
+      </c>
+      <c r="J21" s="14" t="n">
+        <v>119000</v>
+      </c>
+      <c r="K21" s="15">
+        <f>(J21-I21)/J21</f>
+        <v/>
+      </c>
+      <c r="L21" s="14">
+        <f>J21-I21</f>
+        <v/>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O21" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P21" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q21" s="0" t="n">
+        <v>1466</v>
+      </c>
+      <c r="R21" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="S21" s="0" t="n">
+        <v>350</v>
+      </c>
+      <c r="T21" s="0" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U21" s="0" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V21" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="W21" s="0" t="inlineStr">
+        <is>
+          <t>Máscara facial ergonómica y cono nasal para aromaterapia y limpieza.</t>
+        </is>
+      </c>
+      <c r="X21" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y21" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z21" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA21" s="0" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/sauna-facial-inhalador-termico-spa</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="39">
       <c r="A22" s="3" t="inlineStr">
@@ -1813,18 +3178,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C22" s="7" t="n"/>
-      <c r="D22" s="7" t="n"/>
-      <c r="E22" s="8" t="n"/>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="12" t="n"/>
-      <c r="I22" s="14" t="n"/>
-      <c r="J22" s="14" t="n"/>
-      <c r="K22" s="15" t="n"/>
-      <c r="L22" s="14" t="n"/>
-      <c r="M22" s="3" t="n"/>
-      <c r="N22" s="3" t="n"/>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Masajeadores Faciales y Gua Sha LED</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Dispositivo Esculpidor de Rostro y Reductor SkinLift V-Face</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #96165</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>2228164</t>
+        </is>
+      </c>
+      <c r="H22" s="12" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/2228164</t>
+        </is>
+      </c>
+      <c r="I22" s="14" t="n">
+        <v>29000</v>
+      </c>
+      <c r="J22" s="14" t="n">
+        <v>79000</v>
+      </c>
+      <c r="K22" s="15">
+        <f>(J22-I22)/J22</f>
+        <v/>
+      </c>
+      <c r="L22" s="14">
+        <f>J22-I22</f>
+        <v/>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O22" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P22" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q22" s="0" t="n">
+        <v>452</v>
+      </c>
+      <c r="R22" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="S22" s="0" t="n">
+        <v>350</v>
+      </c>
+      <c r="T22" s="0" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U22" s="0" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V22" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="W22" s="0" t="inlineStr">
+        <is>
+          <t>Banda anatómica EMS con fototerapia roja/azul para contorno mandibular.</t>
+        </is>
+      </c>
+      <c r="X22" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y22" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z22" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA22" s="0" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/tonificador-rostro-papada-skinlift</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="39">
       <c r="A23" s="3" t="inlineStr">
@@ -1837,18 +3299,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C23" s="7" t="n"/>
-      <c r="D23" s="7" t="n"/>
-      <c r="E23" s="8" t="n"/>
-      <c r="F23" s="10" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="12" t="n"/>
-      <c r="I23" s="14" t="n"/>
-      <c r="J23" s="14" t="n"/>
-      <c r="K23" s="15" t="n"/>
-      <c r="L23" s="14" t="n"/>
-      <c r="M23" s="3" t="n"/>
-      <c r="N23" s="3" t="n"/>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Cavitación y Reducción Corporal</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Dispositivo Reafirmante Esculpidor Corporal EMS</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #96165</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>2290771</t>
+        </is>
+      </c>
+      <c r="H23" s="12" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/2290771</t>
+        </is>
+      </c>
+      <c r="I23" s="14" t="n">
+        <v>46000</v>
+      </c>
+      <c r="J23" s="14" t="n">
+        <v>119000</v>
+      </c>
+      <c r="K23" s="15">
+        <f>(J23-I23)/J23</f>
+        <v/>
+      </c>
+      <c r="L23" s="14">
+        <f>J23-I23</f>
+        <v/>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N23" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O23" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P23" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q23" s="0" t="n">
+        <v>208</v>
+      </c>
+      <c r="R23" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="S23" s="0" t="n">
+        <v>350</v>
+      </c>
+      <c r="T23" s="0" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U23" s="0" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V23" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="W23" s="0" t="inlineStr">
+        <is>
+          <t>Electroestimulación muscular profunda de alta frecuencia para abdomen y piernas.</t>
+        </is>
+      </c>
+      <c r="X23" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y23" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z23" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA23" s="0" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/esculpidor-tonificador-corporal-ems</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="39">
       <c r="A24" s="3" t="inlineStr">
@@ -1861,18 +3420,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C24" s="7" t="n"/>
-      <c r="D24" s="7" t="n"/>
-      <c r="E24" s="8" t="n"/>
-      <c r="F24" s="10" t="n"/>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="12" t="n"/>
-      <c r="I24" s="14" t="n"/>
-      <c r="J24" s="14" t="n"/>
-      <c r="K24" s="15" t="n"/>
-      <c r="L24" s="14" t="n"/>
-      <c r="M24" s="3" t="n"/>
-      <c r="N24" s="3" t="n"/>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Alta Frecuencia y Microcorrientes</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Masajeador Facial de Microcorrientes Bipolar y Esferas 3D</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #49923</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>2185008</t>
+        </is>
+      </c>
+      <c r="H24" s="12" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/2185008</t>
+        </is>
+      </c>
+      <c r="I24" s="14" t="n">
+        <v>16270</v>
+      </c>
+      <c r="J24" s="14" t="n">
+        <v>59000</v>
+      </c>
+      <c r="K24" s="15">
+        <f>(J24-I24)/J24</f>
+        <v/>
+      </c>
+      <c r="L24" s="14">
+        <f>J24-I24</f>
+        <v/>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N24" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O24" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P24" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q24" s="0" t="n">
+        <v>2688</v>
+      </c>
+      <c r="R24" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="S24" s="0" t="n">
+        <v>350</v>
+      </c>
+      <c r="T24" s="0" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U24" s="0" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V24" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="W24" s="0" t="inlineStr">
+        <is>
+          <t>Esferas giratorias a 70° que reproducen pinzamiento dérmico profesional.</t>
+        </is>
+      </c>
+      <c r="X24" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y24" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z24" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA24" s="0" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/masajeador-microcorriente-esferas-3d</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="39">
       <c r="A25" s="3" t="inlineStr">
@@ -1885,18 +3541,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C25" s="7" t="n"/>
-      <c r="D25" s="7" t="n"/>
-      <c r="E25" s="8" t="n"/>
-      <c r="F25" s="10" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="18" t="n"/>
-      <c r="I25" s="14" t="n"/>
-      <c r="J25" s="14" t="n"/>
-      <c r="K25" s="15" t="n"/>
-      <c r="L25" s="14" t="n"/>
-      <c r="M25" s="3" t="n"/>
-      <c r="N25" s="3" t="n"/>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Extractores de Poros y Succión</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Extractor de Puntos Negros Eléctrico con Pantalla LCD</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #55394</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>339276</t>
+        </is>
+      </c>
+      <c r="H25" s="18" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/339276</t>
+        </is>
+      </c>
+      <c r="I25" s="14" t="n">
+        <v>25000</v>
+      </c>
+      <c r="J25" s="14" t="n">
+        <v>69000</v>
+      </c>
+      <c r="K25" s="15">
+        <f>(J25-I25)/J25</f>
+        <v/>
+      </c>
+      <c r="L25" s="14">
+        <f>J25-I25</f>
+        <v/>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N25" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O25" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P25" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q25" s="0" t="n">
+        <v>124</v>
+      </c>
+      <c r="R25" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="S25" s="0" t="n">
+        <v>350</v>
+      </c>
+      <c r="T25" s="0" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U25" s="0" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V25" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="W25" s="0" t="inlineStr">
+        <is>
+          <t>Pantalla digital LCD con 3 potencias de succión y 5 boquillas ergonómicas.</t>
+        </is>
+      </c>
+      <c r="X25" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y25" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z25" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA25" s="0" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/extractor-puntos-negros-pantalla-lcd</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="39">
       <c r="A26" s="3" t="inlineStr">
@@ -1909,18 +3662,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C26" s="7" t="n"/>
-      <c r="D26" s="7" t="n"/>
-      <c r="E26" s="8" t="n"/>
-      <c r="F26" s="10" t="n"/>
-      <c r="G26" s="3" t="n"/>
-      <c r="H26" s="17" t="n"/>
-      <c r="I26" s="14" t="n"/>
-      <c r="J26" s="14" t="n"/>
-      <c r="K26" s="15" t="n"/>
-      <c r="L26" s="14" t="n"/>
-      <c r="M26" s="3" t="n"/>
-      <c r="N26" s="3" t="n"/>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Cepillos y Limpiadores Sónicos</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Cepillo Limpiador Facial de Drenaje Linfático y Silicona</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #6006</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>2212435</t>
+        </is>
+      </c>
+      <c r="H26" s="17" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/2212435</t>
+        </is>
+      </c>
+      <c r="I26" s="14" t="n">
+        <v>12890</v>
+      </c>
+      <c r="J26" s="14" t="n">
+        <v>49000</v>
+      </c>
+      <c r="K26" s="15">
+        <f>(J26-I26)/J26</f>
+        <v/>
+      </c>
+      <c r="L26" s="14">
+        <f>J26-I26</f>
+        <v/>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N26" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O26" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P26" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q26" s="0" t="n">
+        <v>562</v>
+      </c>
+      <c r="R26" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="S26" s="0" t="n">
+        <v>350</v>
+      </c>
+      <c r="T26" s="0" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U26" s="0" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V26" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="W26" s="0" t="inlineStr">
+        <is>
+          <t>Silicona médica no porosa con reverso estriado para drenaje linfático.</t>
+        </is>
+      </c>
+      <c r="X26" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y26" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z26" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA26" s="0" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/cepillo-facial-drenaje-linfatico</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="39">
       <c r="A27" s="3" t="inlineStr">
@@ -1933,18 +3783,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C27" s="7" t="n"/>
-      <c r="D27" s="7" t="n"/>
-      <c r="E27" s="8" t="n"/>
-      <c r="F27" s="10" t="n"/>
-      <c r="G27" s="3" t="n"/>
-      <c r="H27" s="17" t="n"/>
-      <c r="I27" s="14" t="n"/>
-      <c r="J27" s="14" t="n"/>
-      <c r="K27" s="15" t="n"/>
-      <c r="L27" s="14" t="n"/>
-      <c r="M27" s="3" t="n"/>
-      <c r="N27" s="3" t="n"/>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Dermapen y Microneedling</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Dermapen Inalámbrico Metálico de Alta Precisión</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #325736</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>1474508</t>
+        </is>
+      </c>
+      <c r="H27" s="17" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/1474508</t>
+        </is>
+      </c>
+      <c r="I27" s="14" t="n">
+        <v>112443</v>
+      </c>
+      <c r="J27" s="14" t="n">
+        <v>229000</v>
+      </c>
+      <c r="K27" s="15">
+        <f>(J27-I27)/J27</f>
+        <v/>
+      </c>
+      <c r="L27" s="14">
+        <f>J27-I27</f>
+        <v/>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N27" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O27" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P27" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q27" s="0" t="n">
+        <v>1000</v>
+      </c>
+      <c r="R27" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="S27" s="0" t="n">
+        <v>350</v>
+      </c>
+      <c r="T27" s="0" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U27" s="0" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V27" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="W27" s="0" t="inlineStr">
+        <is>
+          <t>Cuerpo de aluminio aeronáutico y motor de alta estabilidad sin oscilación.</t>
+        </is>
+      </c>
+      <c r="X27" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y27" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z27" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA27" s="0" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/dermapen-inalambrico-metalico-alta-precision</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="39">
       <c r="A28" s="3" t="inlineStr">
@@ -1957,18 +3904,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C28" s="7" t="n"/>
-      <c r="D28" s="7" t="n"/>
-      <c r="E28" s="8" t="n"/>
-      <c r="F28" s="10" t="n"/>
-      <c r="G28" s="3" t="n"/>
-      <c r="H28" s="24" t="n"/>
-      <c r="I28" s="14" t="n"/>
-      <c r="J28" s="14" t="n"/>
-      <c r="K28" s="15" t="n"/>
-      <c r="L28" s="14" t="n"/>
-      <c r="M28" s="3" t="n"/>
-      <c r="N28" s="3" t="n"/>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Radiofrecuencia y Electroporación</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Aparato de Electroporación y Mesoterapia Virtual Transdérmica</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #13615</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>340169</t>
+        </is>
+      </c>
+      <c r="H28" s="24" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/340169</t>
+        </is>
+      </c>
+      <c r="I28" s="14" t="n">
+        <v>45900</v>
+      </c>
+      <c r="J28" s="14" t="n">
+        <v>129000</v>
+      </c>
+      <c r="K28" s="15">
+        <f>(J28-I28)/J28</f>
+        <v/>
+      </c>
+      <c r="L28" s="14">
+        <f>J28-I28</f>
+        <v/>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O28" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P28" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q28" s="0" t="n">
+        <v>93</v>
+      </c>
+      <c r="R28" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="S28" s="0" t="n">
+        <v>350</v>
+      </c>
+      <c r="T28" s="0" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U28" s="0" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V28" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="W28" s="0" t="inlineStr">
+        <is>
+          <t>Permeabilidad transmembrana para absorción de principios activos sin aguja.</t>
+        </is>
+      </c>
+      <c r="X28" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y28" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z28" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA28" s="0" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/electroporacion-mesoterapia-virtual-transdermica</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="39">
       <c r="A29" s="3" t="inlineStr">
@@ -1981,18 +4025,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C29" s="7" t="n"/>
-      <c r="D29" s="7" t="n"/>
-      <c r="E29" s="8" t="n"/>
-      <c r="F29" s="10" t="n"/>
-      <c r="G29" s="3" t="n"/>
-      <c r="H29" s="17" t="n"/>
-      <c r="I29" s="14" t="n"/>
-      <c r="J29" s="14" t="n"/>
-      <c r="K29" s="15" t="n"/>
-      <c r="L29" s="14" t="n"/>
-      <c r="M29" s="3" t="n"/>
-      <c r="N29" s="3" t="n"/>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Vaporizadores y Saunas Faciales</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Vaporizador Facial Portátil Nano-Mister Recargable</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #651557</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>2281692</t>
+        </is>
+      </c>
+      <c r="H29" s="17" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/2281692</t>
+        </is>
+      </c>
+      <c r="I29" s="14" t="n">
+        <v>12000</v>
+      </c>
+      <c r="J29" s="14" t="n">
+        <v>39000</v>
+      </c>
+      <c r="K29" s="15">
+        <f>(J29-I29)/J29</f>
+        <v/>
+      </c>
+      <c r="L29" s="14">
+        <f>J29-I29</f>
+        <v/>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N29" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O29" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P29" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q29" s="0" t="n">
+        <v>200</v>
+      </c>
+      <c r="R29" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="S29" s="0" t="n">
+        <v>350</v>
+      </c>
+      <c r="T29" s="0" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U29" s="0" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V29" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="W29" s="0" t="inlineStr">
+        <is>
+          <t>Atomización ultrasónica de bolsillo para hidratación y fijación de maquillaje.</t>
+        </is>
+      </c>
+      <c r="X29" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y29" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z29" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA29" s="0" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/vaporizador-portatil-nano-mister-recargable</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="39">
       <c r="A30" s="3" t="inlineStr">
@@ -2005,18 +4146,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C30" s="7" t="n"/>
-      <c r="D30" s="7" t="n"/>
-      <c r="E30" s="8" t="n"/>
-      <c r="F30" s="10" t="n"/>
-      <c r="G30" s="3" t="n"/>
-      <c r="H30" s="12" t="n"/>
-      <c r="I30" s="14" t="n"/>
-      <c r="J30" s="14" t="n"/>
-      <c r="K30" s="15" t="n"/>
-      <c r="L30" s="14" t="n"/>
-      <c r="M30" s="3" t="n"/>
-      <c r="N30" s="3" t="n"/>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Alta Frecuencia y Microcorrientes</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Dispositivo Rejuvenecedor Bio-Microcorriente con Rodillos 3D</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #28386</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>2198990</t>
+        </is>
+      </c>
+      <c r="H30" s="12" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/2198990</t>
+        </is>
+      </c>
+      <c r="I30" s="14" t="n">
+        <v>13000</v>
+      </c>
+      <c r="J30" s="14" t="n">
+        <v>49000</v>
+      </c>
+      <c r="K30" s="15">
+        <f>(J30-I30)/J30</f>
+        <v/>
+      </c>
+      <c r="L30" s="14">
+        <f>J30-I30</f>
+        <v/>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N30" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O30" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P30" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q30" s="0" t="n">
+        <v>299</v>
+      </c>
+      <c r="R30" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="S30" s="0" t="n">
+        <v>350</v>
+      </c>
+      <c r="T30" s="0" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U30" s="0" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V30" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="W30" s="0" t="inlineStr">
+        <is>
+          <t>Panel solar captador de luz ambiental que genera bio-microcorrientes continuas.</t>
+        </is>
+      </c>
+      <c r="X30" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y30" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z30" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA30" s="0" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/rejuvenecedor-bio-microcorriente-rodillos-3d</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="39">
       <c r="A31" s="3" t="inlineStr">
@@ -2029,18 +4267,115 @@
           <t>✅ Aprobado</t>
         </is>
       </c>
-      <c r="C31" s="7" t="n"/>
-      <c r="D31" s="7" t="n"/>
-      <c r="E31" s="8" t="n"/>
-      <c r="F31" s="10" t="n"/>
-      <c r="G31" s="3" t="n"/>
-      <c r="H31" s="17" t="n"/>
-      <c r="I31" s="14" t="n"/>
-      <c r="J31" s="14" t="n"/>
-      <c r="K31" s="15" t="n"/>
-      <c r="L31" s="14" t="n"/>
-      <c r="M31" s="3" t="n"/>
-      <c r="N31" s="3" t="n"/>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Beauty Tech</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Masajeadores Faciales y Gua Sha LED</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Ejercitador Mandibular y Perfilador de Mentón Grado Médico</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>Proveedor Verificado #36082</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>2194593</t>
+        </is>
+      </c>
+      <c r="H31" s="17" t="inlineStr">
+        <is>
+          <t>https://app.dropi.co/products/2194593</t>
+        </is>
+      </c>
+      <c r="I31" s="14" t="n">
+        <v>18000</v>
+      </c>
+      <c r="J31" s="14" t="n">
+        <v>49000</v>
+      </c>
+      <c r="K31" s="15">
+        <f>(J31-I31)/J31</f>
+        <v/>
+      </c>
+      <c r="L31" s="14">
+        <f>J31-I31</f>
+        <v/>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sí</t>
+        </is>
+      </c>
+      <c r="N31" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O31" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="P31" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q31" s="0" t="n">
+        <v>499</v>
+      </c>
+      <c r="R31" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="S31" s="0" t="n">
+        <v>350</v>
+      </c>
+      <c r="T31" s="0" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="U31" s="0" t="inlineStr">
+        <is>
+          <t>📈 Subiendo</t>
+        </is>
+      </c>
+      <c r="V31" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="W31" s="0" t="inlineStr">
+        <is>
+          <t>Silicona biocompatible de 30-50 lbs para tonificación del músculo masetero.</t>
+        </is>
+      </c>
+      <c r="X31" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="Y31" s="0" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z31" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="AA31" s="0" t="inlineStr">
+        <is>
+          <t>https://mesolabpro.com.co/producto/ejercitador-mandibular-perfilador-menton</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="39">
       <c r="A32" s="3" t="inlineStr">
@@ -8269,7 +10604,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J19"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="20" customWidth="1" style="39" min="1" max="10"/>
     <col width="8.710000000000001" customWidth="1" style="39" min="11" max="26"/>
@@ -9511,7 +11846,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="35" customWidth="1" style="39" min="1" max="1"/>
     <col width="12" customWidth="1" style="39" min="2" max="2"/>
@@ -10894,7 +13229,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="35" customWidth="1" style="39" min="1" max="1"/>
     <col width="25" customWidth="1" style="39" min="2" max="2"/>
@@ -12116,7 +14451,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8" customWidth="1" style="39" min="1" max="1"/>
     <col width="20" customWidth="1" style="39" min="2" max="2"/>
@@ -13326,7 +15661,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Z1005"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="26.14" customWidth="1" style="39" min="1" max="1"/>
     <col width="29.71" customWidth="1" style="39" min="2" max="2"/>

</xml_diff>